<commit_message>
Preparar entrega final y presentacion de defensa
</commit_message>
<xml_diff>
--- a/docs/video/agora-solicitudes-demo.xlsx
+++ b/docs/video/agora-solicitudes-demo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lourd\Desktop\TFG - Agora\docs\video\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B520E030-31B7-4BA7-BB4C-C6D95FA8662A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B41BAE5D-FF8F-48DB-B000-AF7012DEEFF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11040" xr2:uid="{BA1A631F-4DDF-431D-AA82-92081F0C51C8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20640" windowHeight="11040" xr2:uid="{63209DDB-1C4F-4B6F-9777-CF277E2115EE}"/>
   </bookViews>
   <sheets>
     <sheet name="Solicitudes CSV" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="26">
   <si>
     <t>ID</t>
   </si>
@@ -56,10 +56,10 @@
     <t>Aprobada</t>
   </si>
   <si>
-    <t>Empresa E2E 1774816472977</t>
-  </si>
-  <si>
-    <t>e2e-1774816472977@example.com</t>
+    <t>Empresa demo 01</t>
+  </si>
+  <si>
+    <t>empresa01@demo.local</t>
   </si>
   <si>
     <t>pendiente</t>
@@ -68,40 +68,49 @@
     <t>-</t>
   </si>
   <si>
-    <t>Empresa E2E 1774816179992</t>
-  </si>
-  <si>
-    <t>e2e-1774816179992@example.com</t>
-  </si>
-  <si>
-    <t>Empresa E2E 1774815640882</t>
-  </si>
-  <si>
-    <t>e2e-1774815640882@example.com</t>
-  </si>
-  <si>
-    <t>Verificacion sync 203544</t>
-  </si>
-  <si>
-    <t>lmendezgsd@gmail.com</t>
+    <t>Empresa demo 02</t>
+  </si>
+  <si>
+    <t>empresa02@demo.local</t>
+  </si>
+  <si>
+    <t>Empresa demo 03</t>
+  </si>
+  <si>
+    <t>empresa03@demo.local</t>
+  </si>
+  <si>
+    <t>Empresa demo 04</t>
+  </si>
+  <si>
+    <t>empresa04@demo.local</t>
+  </si>
+  <si>
+    <t>Empresa demo 05</t>
+  </si>
+  <si>
+    <t>empresa05@demo.local</t>
   </si>
   <si>
     <t>aprobada</t>
   </si>
   <si>
-    <t>Prueba Portal Externo 203243</t>
-  </si>
-  <si>
-    <t>Prueba entrega Brevo</t>
-  </si>
-  <si>
-    <t>luisito</t>
-  </si>
-  <si>
-    <t>Empresa E2E 1774807728221</t>
-  </si>
-  <si>
-    <t>e2e-1774807728221@example.com</t>
+    <t>Empresa demo 06</t>
+  </si>
+  <si>
+    <t>empresa06@demo.local</t>
+  </si>
+  <si>
+    <t>Empresa demo 07</t>
+  </si>
+  <si>
+    <t>empresa07@demo.local</t>
+  </si>
+  <si>
+    <t>Empresa demo 08</t>
+  </si>
+  <si>
+    <t>empresa08@demo.local</t>
   </si>
   <si>
     <t>Vista ordenada para la defensa: exportacion CSV abierta como hoja de calculo.</t>
@@ -546,7 +555,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4494550-5F80-44C9-8CE7-EC187F43E170}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D9583614-824C-4C21-87E2-91FB7582B2C2}">
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -579,7 +588,7 @@
     </row>
     <row r="2" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>6</v>
@@ -591,7 +600,7 @@
         <v>8</v>
       </c>
       <c r="E2" s="3">
-        <v>46110.940694444442</v>
+        <v>46124.823460648149</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>9</v>
@@ -599,7 +608,7 @@
     </row>
     <row r="3" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>10</v>
@@ -611,7 +620,7 @@
         <v>8</v>
       </c>
       <c r="E3" s="5">
-        <v>46110.937291666669</v>
+        <v>46110.940694444442</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>9</v>
@@ -619,7 +628,7 @@
     </row>
     <row r="4" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>12</v>
@@ -631,7 +640,7 @@
         <v>8</v>
       </c>
       <c r="E4" s="3">
-        <v>46110.93105324074</v>
+        <v>46110.937291666669</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>9</v>
@@ -639,7 +648,7 @@
     </row>
     <row r="5" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>14</v>
@@ -648,98 +657,98 @@
         <v>15</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E5" s="5">
-        <v>46110.858159722222</v>
-      </c>
-      <c r="F5" s="5">
-        <v>46110.864305555559</v>
+        <v>46110.93105324074</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
+        <v>17</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>15</v>
-      </c>
       <c r="D6" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E6" s="3">
-        <v>46110.856076388889</v>
+        <v>46110.858159722222</v>
       </c>
       <c r="F6" s="3">
-        <v>46110.866157407407</v>
+        <v>46110.864305555559</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>16</v>
-      </c>
       <c r="E7" s="5">
-        <v>46110.853842592594</v>
+        <v>46110.856076388889</v>
       </c>
       <c r="F7" s="5">
-        <v>46110.866180555553</v>
+        <v>46110.866157407407</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E8" s="3">
-        <v>46110.848449074074</v>
+        <v>46110.853842592594</v>
       </c>
       <c r="F8" s="3">
-        <v>46110.866203703707</v>
+        <v>46110.866180555553</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E9" s="5">
-        <v>46110.839479166665</v>
+        <v>46110.848449074074</v>
       </c>
       <c r="F9" s="5">
-        <v>46110.866296296299</v>
+        <v>46110.866203703707</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B11" s="6"/>
       <c r="C11" s="6"/>

</xml_diff>